<commit_message>
Update IO Schedule: EL1859 now includes 3 digital inputs moved from EL1409
EL1859 (Card 10) allocations finalized:
- DO 1-2: Temp Cab Start/Stop (relays on 37-way pins 13, 14)
- DI 1: Temp Cab Run Feedback (latch aux, 37-way pin 15)
- DI 2-4: Pneumatic Open Position, Pneumatic Close Position, E-Stop (moved from EL1409 CH1-3)
- DI 5-8: Spare

EL1409 channels 1-3 marked as relocated to EL1859 in IO Schedule.

Hardware swap sequence confirmed with Jason:
1. Swap EL2869 and EL1409 positions
2. Place EL1859 at end of bus (after EL2869)
3. Connect 3 input wires from EL1409 to EL1859 DI terminals
</commit_message>
<xml_diff>
--- a/commissioning of temperature cabinets/IO_Schedule.xlsx
+++ b/commissioning of temperature cabinets/IO_Schedule.xlsx
@@ -3533,7 +3533,7 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>Pneumtic Open Position</t>
+          <t>Pneumatic Open Position (MOVED TO EL1859 DI 2)</t>
         </is>
       </c>
       <c r="E4" s="1" t="n"/>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>Pneumtic Close Position</t>
+          <t>Pneumatic Close Position (MOVED TO EL1859 DI 3)</t>
         </is>
       </c>
       <c r="E5" s="1" t="n"/>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">E-Stop </t>
+          <t>E-Stop (MOVED TO EL1859 DI 4)</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
@@ -4455,7 +4455,7 @@
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>Spare</t>
+          <t>Pneumatic Open Position</t>
         </is>
       </c>
       <c r="E12" s="1" t="n"/>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>Spare</t>
+          <t>Pneumatic Close Position</t>
         </is>
       </c>
       <c r="E13" s="1" t="n"/>
@@ -4487,10 +4487,14 @@
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>Spare</t>
-        </is>
-      </c>
-      <c r="E14" s="1" t="n"/>
+          <t>E-Stop</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="1" t="n">
@@ -4498,7 +4502,7 @@
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>DI 5</t>
+          <t>DI 4</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
@@ -4514,7 +4518,7 @@
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>DI 6</t>
+          <t>DI 5</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
@@ -4530,7 +4534,7 @@
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>DI 7</t>
+          <t>DI 6</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
@@ -4546,7 +4550,7 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>DI 8</t>
+          <t>DI 7</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">

</xml_diff>